<commit_message>
Actualizacao dados da feira
</commit_message>
<xml_diff>
--- a/Qualidade_Mentoria.xlsx
+++ b/Qualidade_Mentoria.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -414,7 +414,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -424,17 +424,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>RAMIANE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Sessão_4</t>
+          <t>Sessão_6</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Zito Josias</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>15-Jul-2026</t>
+          <t>11-Aug-2026</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>3918786000010652028</t>
+          <t>3918786000010823052</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -481,12 +481,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MUELEGE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Sessão_4</t>
+          <t>Sessão_6</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -501,17 +501,17 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>16-Jul-2026</t>
+          <t>11-Aug-2026</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>3918786000010640095</t>
+          <t>3918786000010813084</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -538,17 +538,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MONAPO RIO</t>
+          <t>MESEREPANE</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sessão_4</t>
+          <t>Sessão_5</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Zito Josias</t>
+          <t>Sergio Fausto</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -558,17 +558,17 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>14-Jul-2026</t>
+          <t>07-Aug-2026</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>3918786000010639055</t>
+          <t>3918786000010801002</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -585,7 +585,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MESEREPANE</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Sergio Fausto</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -615,17 +615,17 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>14-Jul-2026</t>
+          <t>07-Aug-2026</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>3918786000010638034</t>
+          <t>3918786000010800002</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -642,7 +642,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -652,17 +652,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MESEREPANE</t>
+          <t>MUELEGE</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_5</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Sergio Fausto</t>
+          <t>Costa Marques</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -672,17 +672,17 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>02-Jul-2026</t>
+          <t>31-Jul-2026</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>3918786000010611006</t>
+          <t>3918786000010798002</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -699,7 +699,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -709,17 +709,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MESEREPANE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_5</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Sergio Fausto</t>
+          <t>Costa Marques</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -729,17 +729,17 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>18-Jun-2026</t>
+          <t>31-Jul-2026</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>3918786000010611004</t>
+          <t>3918786000010792184</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -756,7 +756,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -766,37 +766,37 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MESEREPANE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_5</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Sergio Fausto</t>
+          <t>Paulo Alexandre</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>04-Jun-2026</t>
+          <t>29-Jul-2026</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>3918786000010611002</t>
+          <t>3918786000010771004</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -813,7 +813,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -828,7 +828,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -838,22 +838,22 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>17-Jun-2026</t>
+          <t>16-Jul-2026</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>3918786000010579063</t>
+          <t>3918786000010771002</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -870,7 +870,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -880,37 +880,37 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>RAMIANE</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_5</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Paulo Alexandre</t>
+          <t>Costa Marques</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>03-Jun-2026</t>
+          <t>30-Jul-2026</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>3918786000010579061</t>
+          <t>3918786000010755028</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -927,7 +927,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -937,17 +937,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_5</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Paulo Alexandre</t>
+          <t>Zito Josias</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -957,17 +957,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>02-Jul-2026</t>
+          <t>28-Jul-2026</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>3918786000010579059</t>
+          <t>3918786000010754002</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -984,7 +984,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -994,12 +994,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MUELEGE</t>
+          <t>RAMIANE</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1014,17 +1014,17 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>18-Jun-2026</t>
+          <t>15-Jul-2026</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>3918786000010573006</t>
+          <t>3918786000010652028</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1041,7 +1041,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1071,17 +1071,17 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>02-Jul-2026</t>
+          <t>16-Jul-2026</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>3918786000010555084</t>
+          <t>3918786000010640095</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1098,7 +1098,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1108,17 +1108,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Zito Josias</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1128,17 +1128,17 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>02-Jul-2026</t>
+          <t>14-Jul-2026</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>3918786000010555030</t>
+          <t>3918786000010639055</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1155,7 +1155,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1165,17 +1165,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MONAPO RIO</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Zito Josias</t>
+          <t>Costa Marques</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1185,17 +1185,17 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>30-Jun-2026</t>
+          <t>14-Jul-2026</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>3918786000010552123</t>
+          <t>3918786000010638034</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1222,17 +1222,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MONAPO RIO</t>
+          <t>MESEREPANE</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Zito Josias</t>
+          <t>Sergio Fausto</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1242,17 +1242,17 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>19-Jun-2026</t>
+          <t>02-Jul-2026</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>3918786000010552121</t>
+          <t>3918786000010611006</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1279,17 +1279,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MONAPO RIO</t>
+          <t>MESEREPANE</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_2</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Zito Josias</t>
+          <t>Sergio Fausto</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1299,17 +1299,17 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>04-Jun-2026</t>
+          <t>18-Jun-2026</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>3918786000010552119</t>
+          <t>3918786000010611004</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1336,17 +1336,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>RAMIANE</t>
+          <t>MESEREPANE</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Sergio Fausto</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1356,17 +1356,17 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>01-Jul-2026</t>
+          <t>04-Jun-2026</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>3918786000010538052</t>
+          <t>3918786000010611002</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1393,42 +1393,42 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MOCONE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_2</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Belo Simao</t>
+          <t>Paulo Alexandre</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>02-Jun-2026</t>
+          <t>17-Jun-2026</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>3918786000010422028</t>
+          <t>3918786000010579063</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Nacala Porto</t>
+          <t>Monapo</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1440,7 +1440,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1455,32 +1455,32 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Otilia Passiel</t>
+          <t>Paulo Alexandre</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>17-Jun-2026</t>
+          <t>03-Jun-2026</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>3918786000010407006</t>
+          <t>3918786000010579061</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1497,7 +1497,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1507,17 +1507,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>RAMIANE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Paulo Alexandre</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1527,17 +1527,17 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>17-Jun-2026</t>
+          <t>02-Jul-2026</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>3918786000010405032</t>
+          <t>3918786000010579059</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1554,7 +1554,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MUELEGE</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1584,17 +1584,17 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>16-Jun-2026</t>
+          <t>18-Jun-2026</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>3918786000010405030</t>
+          <t>3918786000010573006</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1611,7 +1611,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1641,17 +1641,17 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>05-Jun-2026</t>
+          <t>02-Jul-2026</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>3918786000010405028</t>
+          <t>3918786000010555084</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1668,7 +1668,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1678,12 +1678,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>RAMIANE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1698,17 +1698,17 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>04-Jun-2026</t>
+          <t>02-Jul-2026</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>3918786000010405026</t>
+          <t>3918786000010555030</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1725,55 +1725,625 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MONAPO RIO</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Sessão_3</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Zito Josias</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>30-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>3918786000010552123</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>MONAPO RIO</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Sessão_2</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Zito Josias</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>19-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>3918786000010552121</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>MONAPO RIO</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Sessão_1</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Zito Josias</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>04-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>3918786000010552119</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>RAMIANE</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Sessão_3</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>01-Jul-2026</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>3918786000010538052</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>MOCONE</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Sessão_1</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Belo Simao</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>02-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>3918786000010422028</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Nacala Porto</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
         <is>
           <t>TOPELANE</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Sessão_2</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Otilia Passiel</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>17-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>3918786000010407006</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>RAMIANE</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Sessão_2</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>17-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>3918786000010405032</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>TOPELANE</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Sessão_2</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>16-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>3918786000010405030</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>MUELEGE</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
         <is>
           <t>Sessão_1</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>05-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>3918786000010405028</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>RAMIANE</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Sessão_1</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>04-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>3918786000010405026</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>TOPELANE</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Sessão_1</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
         <is>
           <t>03-Jun-2026</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H35" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>3918786000010320010</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>Monapo</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -2040,13 +2610,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0CB5FC74-FE1B-4CE2-9ECF-B166B895D337}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B93C6EED-9DC5-4C78-95AE-EBA9F855ABF6}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E40DC22-366C-4CDF-BDBD-24E5CA416FD3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BAD1A41D-4912-402A-B7FE-BAA28394014A}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FAA5341-359B-4C9A-B801-401C4130D55B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{682CE325-8999-4D5F-BCD3-22093475AFC9}"/>
 </file>
</xml_diff>

<commit_message>
Alteracao das Boxes das feiras
</commit_message>
<xml_diff>
--- a/Qualidade_Mentoria.xlsx
+++ b/Qualidade_Mentoria.xlsx
@@ -2610,13 +2610,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B93C6EED-9DC5-4C78-95AE-EBA9F855ABF6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D929AFA-F9CB-47EB-A6A6-CE3DAF0C9478}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BAD1A41D-4912-402A-B7FE-BAA28394014A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C4CF788D-972F-4CEE-9990-45A122EC8545}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{682CE325-8999-4D5F-BCD3-22093475AFC9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CC660DC8-DB50-4E0F-B04F-2A9299EE1290}"/>
 </file>
</xml_diff>

<commit_message>
Actualizacao dados das feiras
</commit_message>
<xml_diff>
--- a/Qualidade_Mentoria.xlsx
+++ b/Qualidade_Mentoria.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -424,7 +424,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MONAPO RIO</t>
+          <t>MESEREPANE</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -434,7 +434,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Zito Josias</t>
+          <t>Sergio Fausto</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -444,17 +444,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>11-Aug-2026</t>
+          <t>13-Aug-2026</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>3918786000010823052</t>
+          <t>3918786000010849002</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -471,7 +471,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -486,32 +486,32 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Sessão_6</t>
+          <t>Sessão_5</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Paulo Alexandre</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>11-Aug-2026</t>
+          <t>29-Jul-2026</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>3918786000010813084</t>
+          <t>3918786000010844058</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -528,7 +528,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -538,17 +538,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MESEREPANE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Sessão_5</t>
+          <t>Sessão_6</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Sergio Fausto</t>
+          <t>Paulo Alexandre</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -558,17 +558,17 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>07-Aug-2026</t>
+          <t>12-Aug-2026</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>3918786000010801002</t>
+          <t>3918786000010844056</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -585,7 +585,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -595,17 +595,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MESEREPANE</t>
+          <t>MUELEGE</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Sessão_4</t>
+          <t>Sessão_6</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Sergio Fausto</t>
+          <t>Costa Marques</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -615,17 +615,17 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>07-Aug-2026</t>
+          <t>13-Aug-2026</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>3918786000010800002</t>
+          <t>3918786000010839072</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -652,12 +652,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MUELEGE</t>
+          <t>RAMIANE</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sessão_5</t>
+          <t>Sessão_6</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -672,17 +672,17 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>31-Jul-2026</t>
+          <t>13-Aug-2026</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>3918786000010798002</t>
+          <t>3918786000010839002</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -699,7 +699,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -709,17 +709,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Sessão_5</t>
+          <t>Sessão_6</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Zito Josias</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -729,17 +729,17 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>31-Jul-2026</t>
+          <t>11-Aug-2026</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>3918786000010792184</t>
+          <t>3918786000010823052</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -756,7 +756,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -771,32 +771,32 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Sessão_5</t>
+          <t>Sessão_6</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Paulo Alexandre</t>
+          <t>Costa Marques</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>29-Jul-2026</t>
+          <t>11-Aug-2026</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>3918786000010771004</t>
+          <t>3918786000010813084</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -813,7 +813,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -823,17 +823,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MESEREPANE</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Sessão_4</t>
+          <t>Sessão_5</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Paulo Alexandre</t>
+          <t>Sergio Fausto</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -843,17 +843,17 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>16-Jul-2026</t>
+          <t>07-Aug-2026</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>3918786000010771002</t>
+          <t>3918786000010801002</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -870,7 +870,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -880,17 +880,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>RAMIANE</t>
+          <t>MESEREPANE</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Sessão_5</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Sergio Fausto</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -900,17 +900,17 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>30-Jul-2026</t>
+          <t>07-Aug-2026</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>3918786000010755028</t>
+          <t>3918786000010800002</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -927,7 +927,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -937,7 +937,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MONAPO RIO</t>
+          <t>MUELEGE</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Zito Josias</t>
+          <t>Costa Marques</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -957,17 +957,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>28-Jul-2026</t>
+          <t>31-Jul-2026</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>3918786000010754002</t>
+          <t>3918786000010798002</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -984,7 +984,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -994,12 +994,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>RAMIANE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sessão_4</t>
+          <t>Sessão_5</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1014,17 +1014,17 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>15-Jul-2026</t>
+          <t>31-Jul-2026</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>3918786000010652028</t>
+          <t>3918786000010792184</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1041,7 +1041,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1051,37 +1051,37 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MUELEGE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Sessão_4</t>
+          <t>Sessão_5</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Paulo Alexandre</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>16-Jul-2026</t>
+          <t>29-Jul-2026</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>3918786000010640095</t>
+          <t>3918786000010771004</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1098,7 +1098,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MONAPO RIO</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Zito Josias</t>
+          <t>Paulo Alexandre</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1128,17 +1128,17 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>14-Jul-2026</t>
+          <t>16-Jul-2026</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>3918786000010639055</t>
+          <t>3918786000010771002</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1155,7 +1155,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1165,12 +1165,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>RAMIANE</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Sessão_4</t>
+          <t>Sessão_5</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1185,17 +1185,17 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>14-Jul-2026</t>
+          <t>30-Jul-2026</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>3918786000010638034</t>
+          <t>3918786000010755028</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1222,17 +1222,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MESEREPANE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_5</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sergio Fausto</t>
+          <t>Zito Josias</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1242,17 +1242,17 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>02-Jul-2026</t>
+          <t>28-Jul-2026</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>3918786000010611006</t>
+          <t>3918786000010754002</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1269,7 +1269,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1279,17 +1279,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MESEREPANE</t>
+          <t>RAMIANE</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Sergio Fausto</t>
+          <t>Costa Marques</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1299,17 +1299,17 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>18-Jun-2026</t>
+          <t>15-Jul-2026</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>3918786000010611004</t>
+          <t>3918786000010652028</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1326,7 +1326,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1336,17 +1336,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MESEREPANE</t>
+          <t>MUELEGE</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Sergio Fausto</t>
+          <t>Costa Marques</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1356,17 +1356,17 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>04-Jun-2026</t>
+          <t>16-Jul-2026</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>3918786000010611002</t>
+          <t>3918786000010640095</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1383,7 +1383,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1393,37 +1393,37 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Paulo Alexandre</t>
+          <t>Zito Josias</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>17-Jun-2026</t>
+          <t>14-Jul-2026</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>3918786000010579063</t>
+          <t>3918786000010639055</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1440,7 +1440,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1455,32 +1455,32 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_4</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Paulo Alexandre</t>
+          <t>Costa Marques</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>03-Jun-2026</t>
+          <t>14-Jul-2026</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>3918786000010579061</t>
+          <t>3918786000010638034</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1497,7 +1497,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MESEREPANE</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Paulo Alexandre</t>
+          <t>Sergio Fausto</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1532,12 +1532,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>3918786000010579059</t>
+          <t>3918786000010611006</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1554,7 +1554,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MUELEGE</t>
+          <t>MESEREPANE</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Sergio Fausto</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1589,12 +1589,12 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>3918786000010573006</t>
+          <t>3918786000010611004</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1611,7 +1611,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1621,17 +1621,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MUELEGE</t>
+          <t>MESEREPANE</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Sergio Fausto</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1641,17 +1641,17 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>02-Jul-2026</t>
+          <t>04-Jun-2026</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>3918786000010555084</t>
+          <t>3918786000010611002</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1668,7 +1668,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1683,32 +1683,32 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_2</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Paulo Alexandre</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>02-Jul-2026</t>
+          <t>17-Jun-2026</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>3918786000010555030</t>
+          <t>3918786000010579063</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1725,7 +1725,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1735,37 +1735,37 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>MONAPO RIO</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Sessão_3</t>
+          <t>Sessão_1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Zito Josias</t>
+          <t>Paulo Alexandre</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>30-Jun-2026</t>
+          <t>03-Jun-2026</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>3918786000010552123</t>
+          <t>3918786000010579061</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1782,7 +1782,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1792,17 +1792,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MONAPO RIO</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Zito Josias</t>
+          <t>Paulo Alexandre</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1812,17 +1812,17 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>19-Jun-2026</t>
+          <t>02-Jul-2026</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>3918786000010552121</t>
+          <t>3918786000010579059</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1839,7 +1839,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1849,17 +1849,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>MONAPO RIO</t>
+          <t>MUELEGE</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_2</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Zito Josias</t>
+          <t>Costa Marques</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1869,17 +1869,17 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>04-Jun-2026</t>
+          <t>18-Jun-2026</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>3918786000010552119</t>
+          <t>3918786000010573006</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -1896,7 +1896,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1906,7 +1906,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>RAMIANE</t>
+          <t>MUELEGE</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1926,17 +1926,17 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>01-Jul-2026</t>
+          <t>02-Jul-2026</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>3918786000010538052</t>
+          <t>3918786000010555084</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -1953,7 +1953,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1963,17 +1963,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MOCONE</t>
+          <t>TOPELANE</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Belo Simao</t>
+          <t>Costa Marques</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1983,22 +1983,22 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>02-Jun-2026</t>
+          <t>02-Jul-2026</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>3918786000010422028</t>
+          <t>3918786000010555030</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Nacala Porto</t>
+          <t>Monapo</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2010,7 +2010,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2020,17 +2020,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Otilia Passiel</t>
+          <t>Zito Josias</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2040,17 +2040,17 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>17-Jun-2026</t>
+          <t>30-Jun-2026</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>3918786000010407006</t>
+          <t>3918786000010552123</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2067,7 +2067,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>RAMIANE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Zito Josias</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2097,17 +2097,17 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>17-Jun-2026</t>
+          <t>19-Jun-2026</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>3918786000010405032</t>
+          <t>3918786000010552121</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2124,7 +2124,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2134,17 +2134,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>TOPELANE</t>
+          <t>MONAPO RIO</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Sessão_2</t>
+          <t>Sessão_1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Zito Josias</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2154,17 +2154,17 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>16-Jun-2026</t>
+          <t>04-Jun-2026</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>3918786000010405030</t>
+          <t>3918786000010552119</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2181,7 +2181,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2191,12 +2191,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MUELEGE</t>
+          <t>RAMIANE</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Sessão_1</t>
+          <t>Sessão_3</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2211,17 +2211,17 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>05-Jun-2026</t>
+          <t>01-Jul-2026</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>3918786000010405028</t>
+          <t>3918786000010538052</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -2248,7 +2248,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>RAMIANE</t>
+          <t>MOCONE</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Costa Marques</t>
+          <t>Belo Simao</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2268,22 +2268,22 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>04-Jun-2026</t>
+          <t>02-Jun-2026</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>3918786000010405026</t>
+          <t>3918786000010422028</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Monapo</t>
+          <t>Nacala Porto</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2295,55 +2295,340 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>TOPELANE</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Sessão_2</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Otilia Passiel</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>17-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>3918786000010407006</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>RAMIANE</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Sessão_2</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>17-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>3918786000010405032</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
         <is>
           <t>TOPELANE</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Sessão_2</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>16-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>3918786000010405030</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>MUELEGE</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
         <is>
           <t>Sessão_1</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>COSTA MARQUES &amp; OTILIA PASSIEL</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>05-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>3918786000010405028</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>RAMIANE</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Sessão_1</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>04-Jun-2026</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>3918786000010405026</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>TOPELANE</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Sessão_1</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Costa Marques</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
         <is>
           <t>03-Jun-2026</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>3918786000010320010</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>Monapo</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr">
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Monapo</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -2610,13 +2895,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D929AFA-F9CB-47EB-A6A6-CE3DAF0C9478}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD229D69-045D-47B0-A238-D3D2541BC257}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C4CF788D-972F-4CEE-9990-45A122EC8545}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{707C22C4-A95B-4F24-8CBD-C24233E52D92}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CC660DC8-DB50-4E0F-B04F-2A9299EE1290}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A99C033-406F-4D34-8C08-A2D9CDC5E42B}"/>
 </file>
</xml_diff>